<commit_message>
removed errors in test codes
</commit_message>
<xml_diff>
--- a/test_automation/Member2_Test_Execution_Results.xlsx
+++ b/test_automation/Member2_Test_Execution_Results.xlsx
@@ -529,14 +529,14 @@
         <v>5</v>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -558,14 +558,14 @@
         <v>6</v>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>

</xml_diff>